<commit_message>
Keep Kantola configuration and harden ERW startup
</commit_message>
<xml_diff>
--- a/v2/T&C_Code/Inputs/ERW_MOD_PARAM_parameters.xlsx
+++ b/v2/T&C_Code/Inputs/ERW_MOD_PARAM_parameters.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3a3938e8dc8ffb04/Yale/TC-SMEW-N/T^0C-SMEW-N v0.9/v2/T^0C_Code/Inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="57" documentId="13_ncr:1_{0B0F0EB4-1128-4629-B675-51A4EEB78CC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9D1F4D36-4D4B-4F33-A2A5-B3DFFC713233}"/>
+  <xr:revisionPtr revIDLastSave="59" documentId="13_ncr:1_{0B0F0EB4-1128-4629-B675-51A4EEB78CC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3A23DF3D-047E-4E53-B745-8BBE5C31AC3B}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13872" tabRatio="569" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3294" yWindow="3294" windowWidth="17280" windowHeight="9984" tabRatio="569" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="MOD_PARAM" sheetId="3" r:id="rId1"/>
     <sheet name="ERW_MOD" sheetId="4" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="191028"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="75">
   <si>
     <t>M_rock_in</t>
   </si>
@@ -117,9 +117,6 @@
     <t>psd_in</t>
   </si>
   <si>
-    <t>Allerton Project, Leicestershire (UK)</t>
-  </si>
-  <si>
     <t>ZR95_L</t>
   </si>
   <si>
@@ -141,15 +138,6 @@
     <t>fX_conc_convention</t>
   </si>
   <si>
-    <t>conc_to_f_CEC</t>
-  </si>
-  <si>
-    <t>clay loam</t>
-  </si>
-  <si>
-    <t>basalt</t>
-  </si>
-  <si>
     <t>Ca_in</t>
   </si>
   <si>
@@ -168,15 +156,9 @@
     <t>rock_filepath</t>
   </si>
   <si>
-    <t>psd.json</t>
-  </si>
-  <si>
     <t>f_CEC_in</t>
   </si>
   <si>
-    <t>Kelland</t>
-  </si>
-  <si>
     <t>Kbot</t>
   </si>
   <si>
@@ -207,18 +189,12 @@
     <t>blueridge_CDF_data.json</t>
   </si>
   <si>
-    <t>Default Dataset</t>
-  </si>
-  <si>
     <t>cc</t>
   </si>
   <si>
     <t>[0 10 50 100 150 200 300 400 600 800 1000 1250 1500 1750 2000 2500 3000 3500 4000 4500 5000]</t>
   </si>
   <si>
-    <t>control</t>
-  </si>
-  <si>
     <t>MOD_PARAM</t>
   </si>
   <si>
@@ -243,27 +219,15 @@
     <t>NumberOfDays</t>
   </si>
   <si>
-    <t>[0 10 20 50 100 150 200 250 300 400 500]</t>
-  </si>
-  <si>
-    <t>MOD_PARAM_General</t>
-  </si>
-  <si>
     <t>PFT_type</t>
   </si>
   <si>
     <t>stature_type</t>
   </si>
   <si>
-    <t>["L"]</t>
-  </si>
-  <si>
     <t>[1]</t>
   </si>
   <si>
-    <t>[68]</t>
-  </si>
-  <si>
     <t>[0 0]</t>
   </si>
   <si>
@@ -292,12 +256,6 @@
   </si>
   <si>
     <t>crop_Lewis</t>
-  </si>
-  <si>
-    <t>["labradorite", "alkali_feldspar", "diopside", "Fe_forsterite"]</t>
-  </si>
-  <si>
-    <t>[0.35, 0.23, 0.1, 0.01]</t>
   </si>
   <si>
     <t>crop_calcite</t>
@@ -310,11 +268,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
-    <numFmt numFmtId="165" formatCode="0.000000"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -336,32 +293,13 @@
       <name val="Consolas"/>
       <family val="3"/>
     </font>
-    <font>
-      <sz val="11"/>
-      <color theme="5"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
-  <fills count="4">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.79998168889431442"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="7">
@@ -442,7 +380,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -465,24 +403,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" quotePrefix="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="1" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="165" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="49" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -492,10 +412,6 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
@@ -508,15 +424,6 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" quotePrefix="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
@@ -802,7 +709,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7CD89003-D51E-46FB-A15B-91DFDAA3BEF6}">
-  <dimension ref="A1:Y14"/>
+  <dimension ref="A1:Y12"/>
   <sheetFormatPr defaultColWidth="8.68359375" defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="9.1015625" style="2" customWidth="1"/>
@@ -835,31 +742,31 @@
       <c r="A1" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="27" t="s">
-        <v>65</v>
-      </c>
-      <c r="C1" s="28" t="s">
+      <c r="B1" s="15" t="s">
+        <v>57</v>
+      </c>
+      <c r="C1" s="16" t="s">
         <v>5</v>
       </c>
-      <c r="D1" s="29" t="s">
+      <c r="D1" s="17" t="s">
         <v>6</v>
       </c>
-      <c r="E1" s="29" t="s">
+      <c r="E1" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="F1" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="G1" s="28" t="s">
-        <v>64</v>
-      </c>
-      <c r="H1" s="29" t="s">
-        <v>67</v>
+      <c r="F1" s="13" t="s">
+        <v>52</v>
+      </c>
+      <c r="G1" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="H1" s="17" t="s">
+        <v>59</v>
       </c>
       <c r="I1" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="J1" s="30" t="s">
+      <c r="J1" s="18" t="s">
         <v>10</v>
       </c>
       <c r="K1" s="6" t="s">
@@ -887,186 +794,162 @@
         <v>8</v>
       </c>
       <c r="S1" s="6" t="s">
-        <v>57</v>
+        <v>50</v>
       </c>
       <c r="T1" s="6" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="U1" s="6" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="V1" s="6" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="W1" s="6" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="X1" s="6" t="s">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="Y1" s="6" t="s">
-        <v>71</v>
+        <v>61</v>
       </c>
     </row>
     <row r="2" spans="1:25" x14ac:dyDescent="0.55000000000000004">
-      <c r="A2" s="31">
-        <v>1</v>
-      </c>
-      <c r="B2" s="25" t="s">
-        <v>26</v>
-      </c>
-      <c r="C2" s="32" t="s">
+      <c r="A2" s="2">
+        <v>3</v>
+      </c>
+      <c r="B2" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="D2" s="31">
-        <v>52.604328000000002</v>
-      </c>
-      <c r="E2" s="31">
-        <v>0.82565900000000003</v>
-      </c>
-      <c r="F2" s="31" t="s">
-        <v>69</v>
-      </c>
-      <c r="G2" s="31">
+      <c r="C2" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="D2" s="9">
+        <v>40.062778000000002</v>
+      </c>
+      <c r="E2" s="2">
+        <v>-88.196111000000002</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="G2" s="2">
         <v>6</v>
       </c>
-      <c r="H2" s="31">
-        <v>121</v>
-      </c>
-      <c r="I2" s="31">
-        <v>2018</v>
-      </c>
-      <c r="J2" s="33">
-        <v>6.6</v>
-      </c>
-      <c r="K2" s="31">
-        <v>1125</v>
-      </c>
-      <c r="L2" s="31">
-        <v>0.318</v>
-      </c>
-      <c r="M2" s="31">
-        <v>0.32800000000000001</v>
-      </c>
-      <c r="N2" s="31">
-        <v>2.1000000000000001E-2</v>
-      </c>
-      <c r="O2" s="26" t="s">
-        <v>68</v>
-      </c>
-      <c r="P2" s="31">
-        <v>500</v>
-      </c>
-      <c r="Q2" s="31">
-        <v>0</v>
-      </c>
-      <c r="R2" s="31" t="s">
-        <v>73</v>
-      </c>
-      <c r="S2" s="31">
-        <v>1</v>
-      </c>
-      <c r="T2" s="31">
-        <v>150</v>
-      </c>
-      <c r="U2" s="31"/>
-      <c r="V2" s="31">
-        <v>1.35</v>
-      </c>
-      <c r="W2" s="31">
-        <v>30</v>
-      </c>
-      <c r="X2" s="31" t="s">
-        <v>74</v>
-      </c>
-      <c r="Y2" s="31" t="s">
-        <v>72</v>
-      </c>
+      <c r="H2" s="2">
+        <v>1825</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="J2" s="19">
+        <v>6.1</v>
+      </c>
+      <c r="K2" s="2">
+        <v>1295</v>
+      </c>
+      <c r="L2" s="2">
+        <v>0.35</v>
+      </c>
+      <c r="M2" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="N2" s="2">
+        <v>2.5000000000000001E-2</v>
+      </c>
+      <c r="O2" s="14" t="s">
+        <v>51</v>
+      </c>
+      <c r="P2" s="2">
+        <v>300</v>
+      </c>
+      <c r="Q2" s="2">
+        <v>1</v>
+      </c>
+      <c r="R2" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="S2" s="2">
+        <v>2</v>
+      </c>
+      <c r="T2"/>
+      <c r="U2"/>
+      <c r="V2"/>
+      <c r="W2"/>
     </row>
     <row r="3" spans="1:25" x14ac:dyDescent="0.55000000000000004">
-      <c r="A3" s="31">
+      <c r="A3" s="2">
+        <v>4</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="D3" s="9">
+        <v>40.062778000000002</v>
+      </c>
+      <c r="E3" s="2">
+        <v>-88.196111000000002</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="G3" s="2">
+        <v>6</v>
+      </c>
+      <c r="H3" s="2">
+        <v>1825</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="J3" s="19">
+        <v>6.1</v>
+      </c>
+      <c r="K3" s="2">
+        <v>1295</v>
+      </c>
+      <c r="L3" s="2">
+        <v>0.35</v>
+      </c>
+      <c r="M3" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="N3" s="2">
+        <v>2.5000000000000001E-2</v>
+      </c>
+      <c r="O3" s="14" t="s">
+        <v>51</v>
+      </c>
+      <c r="P3" s="2">
+        <v>300</v>
+      </c>
+      <c r="Q3" s="2">
+        <v>1</v>
+      </c>
+      <c r="R3" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="S3" s="2">
         <v>2</v>
       </c>
-      <c r="B3" s="25" t="s">
-        <v>26</v>
-      </c>
-      <c r="C3" s="32" t="s">
-        <v>45</v>
-      </c>
-      <c r="D3" s="31">
-        <v>52.604328000000002</v>
-      </c>
-      <c r="E3" s="31">
-        <v>0.82565900000000003</v>
-      </c>
-      <c r="F3" s="31" t="s">
-        <v>69</v>
-      </c>
-      <c r="G3" s="31">
-        <v>6</v>
-      </c>
-      <c r="H3" s="31">
-        <v>121</v>
-      </c>
-      <c r="I3" s="31">
-        <v>2018</v>
-      </c>
-      <c r="J3" s="33">
-        <v>6.6</v>
-      </c>
-      <c r="K3" s="31">
-        <v>1125</v>
-      </c>
-      <c r="L3" s="31">
-        <v>0.318</v>
-      </c>
-      <c r="M3" s="31">
-        <v>0.32800000000000001</v>
-      </c>
-      <c r="N3" s="31">
-        <v>2.1000000000000001E-2</v>
-      </c>
-      <c r="O3" s="26" t="s">
-        <v>68</v>
-      </c>
-      <c r="P3" s="31">
-        <v>500</v>
-      </c>
-      <c r="Q3" s="31">
-        <v>0</v>
-      </c>
-      <c r="R3" s="31" t="s">
-        <v>73</v>
-      </c>
-      <c r="S3" s="31">
-        <v>1</v>
-      </c>
-      <c r="T3" s="31">
-        <v>150</v>
-      </c>
-      <c r="U3" s="31"/>
-      <c r="V3" s="31">
-        <v>1.35</v>
-      </c>
-      <c r="W3" s="31">
-        <v>30</v>
-      </c>
-      <c r="X3" s="31" t="s">
-        <v>74</v>
-      </c>
-      <c r="Y3" s="31" t="s">
-        <v>72</v>
-      </c>
+      <c r="T3"/>
+      <c r="U3"/>
+      <c r="V3"/>
+      <c r="W3"/>
     </row>
     <row r="4" spans="1:25" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="2">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="D4" s="9">
         <v>40.062778000000002</v>
@@ -1075,7 +958,7 @@
         <v>-88.196111000000002</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>61</v>
+        <v>53</v>
       </c>
       <c r="G4" s="2">
         <v>6</v>
@@ -1084,9 +967,9 @@
         <v>1825</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="J4" s="34">
+        <v>66</v>
+      </c>
+      <c r="J4" s="19">
         <v>6.1</v>
       </c>
       <c r="K4" s="2">
@@ -1101,8 +984,8 @@
       <c r="N4" s="2">
         <v>2.5000000000000001E-2</v>
       </c>
-      <c r="O4" s="24" t="s">
-        <v>58</v>
+      <c r="O4" s="14" t="s">
+        <v>51</v>
       </c>
       <c r="P4" s="2">
         <v>300</v>
@@ -1111,7 +994,7 @@
         <v>1</v>
       </c>
       <c r="R4" s="2" t="s">
-        <v>75</v>
+        <v>63</v>
       </c>
       <c r="S4" s="2">
         <v>2</v>
@@ -1123,13 +1006,13 @@
     </row>
     <row r="5" spans="1:25" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="2">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="D5" s="9">
         <v>40.062778000000002</v>
@@ -1138,7 +1021,7 @@
         <v>-88.196111000000002</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>61</v>
+        <v>53</v>
       </c>
       <c r="G5" s="2">
         <v>6</v>
@@ -1147,9 +1030,9 @@
         <v>1825</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="J5" s="34">
+        <v>66</v>
+      </c>
+      <c r="J5" s="19">
         <v>6.1</v>
       </c>
       <c r="K5" s="2">
@@ -1164,8 +1047,8 @@
       <c r="N5" s="2">
         <v>2.5000000000000001E-2</v>
       </c>
-      <c r="O5" s="24" t="s">
-        <v>58</v>
+      <c r="O5" s="14" t="s">
+        <v>51</v>
       </c>
       <c r="P5" s="2">
         <v>300</v>
@@ -1174,7 +1057,7 @@
         <v>1</v>
       </c>
       <c r="R5" s="2" t="s">
-        <v>75</v>
+        <v>63</v>
       </c>
       <c r="S5" s="2">
         <v>2</v>
@@ -1186,13 +1069,13 @@
     </row>
     <row r="6" spans="1:25" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" s="2">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="D6" s="9">
         <v>40.062778000000002</v>
@@ -1201,7 +1084,7 @@
         <v>-88.196111000000002</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>61</v>
+        <v>53</v>
       </c>
       <c r="G6" s="2">
         <v>6</v>
@@ -1210,9 +1093,9 @@
         <v>1825</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="J6" s="34">
+        <v>47</v>
+      </c>
+      <c r="J6" s="19">
         <v>6.1</v>
       </c>
       <c r="K6" s="2">
@@ -1227,8 +1110,8 @@
       <c r="N6" s="2">
         <v>2.5000000000000001E-2</v>
       </c>
-      <c r="O6" s="24" t="s">
-        <v>58</v>
+      <c r="O6" s="14" t="s">
+        <v>51</v>
       </c>
       <c r="P6" s="2">
         <v>300</v>
@@ -1237,7 +1120,7 @@
         <v>1</v>
       </c>
       <c r="R6" s="2" t="s">
-        <v>75</v>
+        <v>63</v>
       </c>
       <c r="S6" s="2">
         <v>2</v>
@@ -1248,145 +1131,19 @@
       <c r="W6"/>
     </row>
     <row r="7" spans="1:25" x14ac:dyDescent="0.55000000000000004">
-      <c r="A7" s="2">
-        <v>6</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="D7" s="9">
-        <v>40.062778000000002</v>
-      </c>
-      <c r="E7" s="2">
-        <v>-88.196111000000002</v>
-      </c>
-      <c r="F7" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="G7" s="2">
-        <v>6</v>
-      </c>
-      <c r="H7" s="2">
-        <v>1825</v>
-      </c>
-      <c r="I7" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="J7" s="34">
-        <v>6.1</v>
-      </c>
-      <c r="K7" s="2">
-        <v>1295</v>
-      </c>
-      <c r="L7" s="2">
-        <v>0.35</v>
-      </c>
-      <c r="M7" s="2">
-        <v>0.1</v>
-      </c>
-      <c r="N7" s="2">
-        <v>2.5000000000000001E-2</v>
-      </c>
-      <c r="O7" s="24" t="s">
-        <v>58</v>
-      </c>
-      <c r="P7" s="2">
-        <v>300</v>
-      </c>
-      <c r="Q7" s="2">
-        <v>1</v>
-      </c>
-      <c r="R7" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="S7" s="2">
-        <v>2</v>
-      </c>
-      <c r="T7"/>
-      <c r="U7"/>
-      <c r="V7"/>
-      <c r="W7"/>
+      <c r="J7"/>
     </row>
     <row r="8" spans="1:25" x14ac:dyDescent="0.55000000000000004">
-      <c r="A8" s="2">
-        <v>7</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="D8" s="9">
-        <v>40.062778000000002</v>
-      </c>
-      <c r="E8" s="2">
-        <v>-88.196111000000002</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="G8" s="2">
-        <v>6</v>
-      </c>
-      <c r="H8" s="2">
-        <v>1825</v>
-      </c>
-      <c r="I8" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="J8" s="34">
-        <v>6.1</v>
-      </c>
-      <c r="K8" s="2">
-        <v>1295</v>
-      </c>
-      <c r="L8" s="2">
-        <v>0.35</v>
-      </c>
-      <c r="M8" s="2">
-        <v>0.1</v>
-      </c>
-      <c r="N8" s="2">
-        <v>2.5000000000000001E-2</v>
-      </c>
-      <c r="O8" s="24" t="s">
-        <v>58</v>
-      </c>
-      <c r="P8" s="2">
-        <v>300</v>
-      </c>
-      <c r="Q8" s="2">
-        <v>1</v>
-      </c>
-      <c r="R8" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="S8" s="2">
-        <v>2</v>
-      </c>
-      <c r="T8"/>
-      <c r="U8"/>
-      <c r="V8"/>
-      <c r="W8"/>
+      <c r="J8"/>
     </row>
     <row r="9" spans="1:25" x14ac:dyDescent="0.55000000000000004">
-      <c r="J9"/>
+      <c r="S9" s="9"/>
     </row>
     <row r="10" spans="1:25" x14ac:dyDescent="0.55000000000000004">
-      <c r="J10"/>
-    </row>
-    <row r="11" spans="1:25" x14ac:dyDescent="0.55000000000000004">
-      <c r="S11" s="9"/>
+      <c r="S10" s="9"/>
     </row>
     <row r="12" spans="1:25" x14ac:dyDescent="0.55000000000000004">
-      <c r="S12" s="9"/>
-    </row>
-    <row r="14" spans="1:25" x14ac:dyDescent="0.55000000000000004">
-      <c r="Q14" s="9"/>
+      <c r="Q12" s="9"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1396,7 +1153,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D139F640-0076-4304-86A9-B1EEDC96C211}">
-  <dimension ref="A1:AH8"/>
+  <dimension ref="A1:AH6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="10.1015625" customWidth="1"/>
@@ -1429,74 +1186,74 @@
       <c r="A1" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="20" t="s">
-        <v>65</v>
-      </c>
-      <c r="C1" s="21" t="s">
+      <c r="B1" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C1" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="D1" s="22" t="s">
+      <c r="D1" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="E1" s="22" t="s">
+      <c r="E1" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="F1" s="23" t="s">
-        <v>66</v>
+      <c r="F1" s="13" t="s">
+        <v>58</v>
       </c>
       <c r="G1" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="H1" s="6" t="s">
-        <v>29</v>
-      </c>
       <c r="I1" s="6" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="J1" s="5" t="s">
         <v>12</v>
       </c>
       <c r="K1" s="5" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="L1" s="5" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="M1" s="5" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="N1" s="5" t="s">
         <v>13</v>
       </c>
       <c r="O1" s="5" t="s">
-        <v>76</v>
+        <v>64</v>
       </c>
       <c r="P1" s="5" t="s">
         <v>21</v>
       </c>
       <c r="Q1" s="5" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="R1" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="S1" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="T1" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="U1" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="V1" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="S1" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="T1" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="U1" s="5" t="s">
+      <c r="W1" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="X1" s="5" t="s">
         <v>39</v>
-      </c>
-      <c r="V1" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="W1" s="5" t="s">
-        <v>40</v>
-      </c>
-      <c r="X1" s="5" t="s">
-        <v>44</v>
       </c>
       <c r="Y1" s="5" t="s">
         <v>0</v>
@@ -1520,7 +1277,7 @@
         <v>22</v>
       </c>
       <c r="AF1" s="5" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="AG1" s="5" t="s">
         <v>2</v>
@@ -1530,196 +1287,176 @@
       </c>
     </row>
     <row r="2" spans="1:34" x14ac:dyDescent="0.55000000000000004">
-      <c r="A2" s="13">
-        <v>1</v>
-      </c>
-      <c r="B2" s="12" t="s">
-        <v>26</v>
-      </c>
-      <c r="C2" s="11" t="s">
+      <c r="A2" s="4">
+        <v>3</v>
+      </c>
+      <c r="B2" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="D2" s="16">
-        <v>52.604328000000002</v>
-      </c>
-      <c r="E2" s="16">
-        <v>0.82565900000000003</v>
-      </c>
-      <c r="F2" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="G2" s="10">
-        <v>1</v>
-      </c>
-      <c r="H2" s="10">
-        <v>1</v>
-      </c>
-      <c r="I2" s="10" t="s">
-        <v>34</v>
-      </c>
-      <c r="J2" s="13">
-        <v>0</v>
-      </c>
-      <c r="K2" s="14" t="s">
-        <v>45</v>
-      </c>
-      <c r="L2" s="14" t="s">
-        <v>43</v>
-      </c>
-      <c r="M2" s="14" t="s">
-        <v>56</v>
-      </c>
-      <c r="N2" s="14" t="s">
-        <v>35</v>
-      </c>
-      <c r="O2" s="17">
-        <v>25.4</v>
-      </c>
-      <c r="P2" s="17">
-        <v>0</v>
-      </c>
-      <c r="Q2" s="17">
-        <v>0</v>
-      </c>
-      <c r="R2" s="17">
+      <c r="C2" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="D2" s="9">
+        <v>40.062778000000002</v>
+      </c>
+      <c r="E2" s="2">
+        <v>-88.196111000000002</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="G2" s="2">
+        <v>1</v>
+      </c>
+      <c r="H2" s="2">
+        <v>1</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="J2" s="4">
+        <v>1</v>
+      </c>
+      <c r="K2" t="s">
+        <v>46</v>
+      </c>
+      <c r="L2" t="s">
+        <v>49</v>
+      </c>
+      <c r="M2" t="s">
+        <v>54</v>
+      </c>
+      <c r="N2" t="s">
+        <v>48</v>
+      </c>
+      <c r="O2" s="7">
+        <v>8.6</v>
+      </c>
+      <c r="P2" s="7">
+        <v>0</v>
+      </c>
+      <c r="Q2" s="7">
+        <v>0</v>
+      </c>
+      <c r="R2" s="7"/>
+      <c r="S2" s="7"/>
+      <c r="T2" s="7"/>
+      <c r="U2" s="7"/>
+      <c r="V2" s="7"/>
+      <c r="W2" s="7"/>
+      <c r="Y2">
+        <v>0</v>
+      </c>
+      <c r="Z2" t="s">
         <v>70</v>
       </c>
-      <c r="S2" s="17">
-        <v>800</v>
-      </c>
-      <c r="T2" s="17">
-        <v>30</v>
-      </c>
-      <c r="U2" s="17">
-        <v>190</v>
-      </c>
-      <c r="V2" s="17">
-        <v>200</v>
-      </c>
-      <c r="W2" s="17">
-        <v>2500</v>
-      </c>
-      <c r="X2" s="15"/>
-      <c r="Y2" s="14">
-        <v>10000</v>
-      </c>
-      <c r="Z2" s="14" t="s">
-        <v>85</v>
-      </c>
-      <c r="AA2" s="18" t="s">
-        <v>86</v>
-      </c>
-      <c r="AB2" s="14">
+      <c r="AA2" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="AB2">
         <f t="shared" ref="AB2:AB3" si="0">3*1000000</f>
         <v>3000000</v>
       </c>
-      <c r="AC2" s="14"/>
-      <c r="AD2" s="14"/>
-      <c r="AE2" s="14">
-        <v>7.35</v>
-      </c>
-      <c r="AF2" s="14">
-        <v>0.8</v>
-      </c>
-      <c r="AG2" s="14">
-        <v>0.5</v>
-      </c>
-      <c r="AH2" s="14">
+      <c r="AE2">
+        <v>1.02</v>
+      </c>
+      <c r="AG2">
+        <v>1</v>
+      </c>
+      <c r="AH2">
         <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:34" x14ac:dyDescent="0.55000000000000004">
-      <c r="A3" s="13">
-        <v>2</v>
-      </c>
-      <c r="B3" s="12" t="s">
-        <v>26</v>
-      </c>
-      <c r="C3" s="11" t="s">
+      <c r="A3" s="4">
+        <v>4</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="D3" s="16">
-        <v>52.604328000000002</v>
-      </c>
-      <c r="E3" s="16">
-        <v>0.82565900000000003</v>
-      </c>
-      <c r="F3" s="10" t="s">
-        <v>59</v>
-      </c>
-      <c r="G3" s="10">
-        <v>1</v>
-      </c>
-      <c r="H3" s="10">
-        <v>1</v>
-      </c>
-      <c r="I3" s="10" t="s">
-        <v>34</v>
-      </c>
-      <c r="J3" s="13">
-        <v>0</v>
-      </c>
-      <c r="K3" s="14"/>
-      <c r="L3" s="14"/>
-      <c r="M3" s="14"/>
-      <c r="N3" s="14" t="s">
-        <v>35</v>
-      </c>
-      <c r="O3" s="17">
-        <v>25.4</v>
-      </c>
-      <c r="P3" s="17">
-        <v>0</v>
-      </c>
-      <c r="Q3" s="17">
-        <v>0</v>
-      </c>
-      <c r="R3" s="17">
-        <v>70</v>
-      </c>
-      <c r="S3" s="17">
-        <v>800</v>
-      </c>
-      <c r="T3" s="17">
-        <v>30</v>
-      </c>
-      <c r="U3" s="17">
-        <v>190</v>
-      </c>
-      <c r="V3" s="17">
-        <v>200</v>
-      </c>
-      <c r="W3" s="17">
-        <v>2500</v>
-      </c>
-      <c r="X3" s="17"/>
-      <c r="Y3" s="14">
-        <v>0</v>
-      </c>
-      <c r="Z3" s="14"/>
-      <c r="AA3" s="14"/>
-      <c r="AB3" s="14">
+      <c r="C3" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="D3" s="9">
+        <v>40.062778000000002</v>
+      </c>
+      <c r="E3" s="2">
+        <v>-88.196111000000002</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="G3" s="2">
+        <v>1</v>
+      </c>
+      <c r="H3" s="2">
+        <v>1</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="J3" s="4">
+        <v>1</v>
+      </c>
+      <c r="K3" t="s">
+        <v>46</v>
+      </c>
+      <c r="L3" t="s">
+        <v>49</v>
+      </c>
+      <c r="M3" t="s">
+        <v>54</v>
+      </c>
+      <c r="N3" t="s">
+        <v>48</v>
+      </c>
+      <c r="O3" s="7">
+        <v>8.6</v>
+      </c>
+      <c r="P3" s="7">
+        <v>0</v>
+      </c>
+      <c r="Q3" s="7">
+        <v>0</v>
+      </c>
+      <c r="R3" s="7"/>
+      <c r="S3" s="7"/>
+      <c r="T3" s="7"/>
+      <c r="U3" s="7"/>
+      <c r="V3" s="7"/>
+      <c r="W3" s="7"/>
+      <c r="Y3">
+        <v>0</v>
+      </c>
+      <c r="Z3" t="s">
+        <v>67</v>
+      </c>
+      <c r="AA3" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="AB3">
         <f t="shared" si="0"/>
         <v>3000000</v>
       </c>
-      <c r="AC3" s="14"/>
-      <c r="AD3" s="14"/>
-      <c r="AE3" s="14"/>
-      <c r="AF3" s="19"/>
-      <c r="AG3" s="14"/>
-      <c r="AH3" s="14">
+      <c r="AE3">
+        <v>1.02</v>
+      </c>
+      <c r="AG3">
+        <v>1</v>
+      </c>
+      <c r="AH3">
         <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:34" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="4">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="D4" s="9">
         <v>40.062778000000002</v>
@@ -1727,8 +1464,8 @@
       <c r="E4" s="2">
         <v>-88.196111000000002</v>
       </c>
-      <c r="F4" s="2" t="s">
-        <v>83</v>
+      <c r="F4" t="s">
+        <v>55</v>
       </c>
       <c r="G4" s="2">
         <v>1</v>
@@ -1737,22 +1474,16 @@
         <v>1</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="J4" s="4">
         <v>1</v>
       </c>
       <c r="K4" t="s">
-        <v>52</v>
-      </c>
-      <c r="L4" t="s">
-        <v>55</v>
-      </c>
-      <c r="M4" t="s">
-        <v>62</v>
+        <v>46</v>
       </c>
       <c r="N4" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="O4" s="7">
         <v>8.6</v>
@@ -1772,35 +1503,20 @@
       <c r="Y4">
         <v>0</v>
       </c>
-      <c r="Z4" t="s">
-        <v>82</v>
-      </c>
-      <c r="AA4" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="AB4">
-        <f t="shared" ref="AB4:AB5" si="1">3*1000000</f>
-        <v>3000000</v>
-      </c>
-      <c r="AE4">
-        <v>1.02</v>
-      </c>
-      <c r="AG4">
-        <v>1</v>
-      </c>
+      <c r="AA4" s="8"/>
       <c r="AH4">
         <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:34" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="4">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="D5" s="9">
         <v>40.062778000000002</v>
@@ -1808,8 +1524,8 @@
       <c r="E5" s="2">
         <v>-88.196111000000002</v>
       </c>
-      <c r="F5" s="2" t="s">
-        <v>84</v>
+      <c r="F5" t="s">
+        <v>65</v>
       </c>
       <c r="G5" s="2">
         <v>1</v>
@@ -1818,22 +1534,16 @@
         <v>1</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="J5" s="4">
         <v>1</v>
       </c>
       <c r="K5" t="s">
-        <v>52</v>
-      </c>
-      <c r="L5" t="s">
-        <v>55</v>
-      </c>
-      <c r="M5" t="s">
-        <v>62</v>
+        <v>46</v>
       </c>
       <c r="N5" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="O5" s="7">
         <v>8.6</v>
@@ -1853,35 +1563,20 @@
       <c r="Y5">
         <v>0</v>
       </c>
-      <c r="Z5" t="s">
-        <v>79</v>
-      </c>
-      <c r="AA5" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="AB5">
-        <f t="shared" si="1"/>
-        <v>3000000</v>
-      </c>
-      <c r="AE5">
-        <v>1.02</v>
-      </c>
-      <c r="AG5">
-        <v>1</v>
-      </c>
+      <c r="AA5" s="8"/>
       <c r="AH5">
         <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:34" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" s="4">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="D6" s="9">
         <v>40.062778000000002</v>
@@ -1889,8 +1584,8 @@
       <c r="E6" s="2">
         <v>-88.196111000000002</v>
       </c>
-      <c r="F6" t="s">
-        <v>63</v>
+      <c r="F6" s="2" t="s">
+        <v>73</v>
       </c>
       <c r="G6" s="2">
         <v>1</v>
@@ -1899,16 +1594,22 @@
         <v>1</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="J6" s="4">
         <v>1</v>
       </c>
       <c r="K6" t="s">
-        <v>52</v>
+        <v>46</v>
+      </c>
+      <c r="L6" t="s">
+        <v>49</v>
+      </c>
+      <c r="M6" t="s">
+        <v>54</v>
       </c>
       <c r="N6" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="O6" s="7">
         <v>8.6</v>
@@ -1928,149 +1629,23 @@
       <c r="Y6">
         <v>0</v>
       </c>
-      <c r="AA6" s="8"/>
+      <c r="Z6" t="s">
+        <v>74</v>
+      </c>
+      <c r="AA6" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="AB6">
+        <f t="shared" ref="AB6" si="1">3*1000000</f>
+        <v>3000000</v>
+      </c>
+      <c r="AE6">
+        <v>1.02</v>
+      </c>
+      <c r="AG6">
+        <v>1</v>
+      </c>
       <c r="AH6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:34" x14ac:dyDescent="0.55000000000000004">
-      <c r="A7" s="4">
-        <v>6</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="D7" s="9">
-        <v>40.062778000000002</v>
-      </c>
-      <c r="E7" s="2">
-        <v>-88.196111000000002</v>
-      </c>
-      <c r="F7" t="s">
-        <v>77</v>
-      </c>
-      <c r="G7" s="2">
-        <v>1</v>
-      </c>
-      <c r="H7" s="2">
-        <v>1</v>
-      </c>
-      <c r="I7" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="J7" s="4">
-        <v>1</v>
-      </c>
-      <c r="K7" t="s">
-        <v>52</v>
-      </c>
-      <c r="N7" t="s">
-        <v>54</v>
-      </c>
-      <c r="O7" s="7">
-        <v>8.6</v>
-      </c>
-      <c r="P7" s="7">
-        <v>0</v>
-      </c>
-      <c r="Q7" s="7">
-        <v>0</v>
-      </c>
-      <c r="R7" s="7"/>
-      <c r="S7" s="7"/>
-      <c r="T7" s="7"/>
-      <c r="U7" s="7"/>
-      <c r="V7" s="7"/>
-      <c r="W7" s="7"/>
-      <c r="Y7">
-        <v>0</v>
-      </c>
-      <c r="AA7" s="8"/>
-      <c r="AH7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:34" x14ac:dyDescent="0.55000000000000004">
-      <c r="A8" s="4">
-        <v>7</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="D8" s="9">
-        <v>40.062778000000002</v>
-      </c>
-      <c r="E8" s="2">
-        <v>-88.196111000000002</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="G8" s="2">
-        <v>1</v>
-      </c>
-      <c r="H8" s="2">
-        <v>1</v>
-      </c>
-      <c r="I8" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="J8" s="4">
-        <v>1</v>
-      </c>
-      <c r="K8" t="s">
-        <v>52</v>
-      </c>
-      <c r="L8" t="s">
-        <v>55</v>
-      </c>
-      <c r="M8" t="s">
-        <v>62</v>
-      </c>
-      <c r="N8" t="s">
-        <v>54</v>
-      </c>
-      <c r="O8" s="7">
-        <v>8.6</v>
-      </c>
-      <c r="P8" s="7">
-        <v>0</v>
-      </c>
-      <c r="Q8" s="7">
-        <v>0</v>
-      </c>
-      <c r="R8" s="7"/>
-      <c r="S8" s="7"/>
-      <c r="T8" s="7"/>
-      <c r="U8" s="7"/>
-      <c r="V8" s="7"/>
-      <c r="W8" s="7"/>
-      <c r="Y8">
-        <v>0</v>
-      </c>
-      <c r="Z8" t="s">
-        <v>88</v>
-      </c>
-      <c r="AA8" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="AB8">
-        <f t="shared" ref="AB8" si="2">3*1000000</f>
-        <v>3000000</v>
-      </c>
-      <c r="AE8">
-        <v>1.02</v>
-      </c>
-      <c r="AG8">
-        <v>1</v>
-      </c>
-      <c r="AH8">
         <v>0</v>
       </c>
     </row>
@@ -2099,15 +1674,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100BA25395398D53143824DAEC78DD9561A" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="20ccdcc7d59f2619f731219bc917c622">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="65a37cd7-3d23-4aec-ad96-417b75cab311" xmlns:ns3="155627c1-0cf9-4357-bbd5-48008c93d75a" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="e26a2ebc3a37e9b8f4c1fbd5093d1833" ns2:_="" ns3:_="">
     <xsd:import namespace="65a37cd7-3d23-4aec-ad96-417b75cab311"/>
@@ -2336,6 +1902,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CA802978-8DC2-44C2-8CFD-840D40C88D7C}">
   <ds:schemaRefs>
@@ -2354,14 +1929,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C4807397-6038-423A-9DD2-E48912B9B2FD}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AAA6EAB6-7EA4-41C9-A63C-13457F927A01}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2378,4 +1945,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C4807397-6038-423A-9DD2-E48912B9B2FD}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Checkpoint Bouchet campaign working tree before pH control-offset investigation
</commit_message>
<xml_diff>
--- a/v2/T&C_Code/Inputs/ERW_MOD_PARAM_parameters.xlsx
+++ b/v2/T&C_Code/Inputs/ERW_MOD_PARAM_parameters.xlsx
@@ -1,26 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3a3938e8dc8ffb04/Yale/TC-SMEW-N/T^0C-SMEW-N v0.9/v2/T^0C_Code/Inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="59" documentId="13_ncr:1_{0B0F0EB4-1128-4629-B675-51A4EEB78CC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3A23DF3D-047E-4E53-B745-8BBE5C31AC3B}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="11_195726565ED4F478434924F23CE2D38DFC40A2D1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{757DE8D6-4EB4-40DF-A2E7-EC62B179152E}"/>
   <bookViews>
-    <workbookView xWindow="3294" yWindow="3294" windowWidth="17280" windowHeight="9984" tabRatio="569" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13872" tabRatio="569" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="MOD_PARAM" sheetId="3" r:id="rId1"/>
-    <sheet name="ERW_MOD" sheetId="4" r:id="rId2"/>
+    <sheet name="MOD_PARAM" sheetId="1" r:id="rId1"/>
+    <sheet name="ERW_MOD" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
@@ -37,234 +34,234 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="76">
+  <si>
+    <t>Number</t>
+  </si>
+  <si>
+    <t>ExperimentFullName</t>
+  </si>
+  <si>
+    <t>Location</t>
+  </si>
+  <si>
+    <t>Lat</t>
+  </si>
+  <si>
+    <t>Lon</t>
+  </si>
+  <si>
+    <t>MOD_PARAM</t>
+  </si>
+  <si>
+    <t>t_res</t>
+  </si>
+  <si>
+    <t>NumberOfDays</t>
+  </si>
+  <si>
+    <t>Year</t>
+  </si>
+  <si>
+    <t>PH</t>
+  </si>
+  <si>
+    <t>rsd</t>
+  </si>
+  <si>
+    <t>Pcla</t>
+  </si>
+  <si>
+    <t>Psan</t>
+  </si>
+  <si>
+    <t>Porg</t>
+  </si>
+  <si>
+    <t>Zs</t>
+  </si>
+  <si>
+    <t>Zbio</t>
+  </si>
+  <si>
+    <t>Cbare</t>
+  </si>
+  <si>
+    <t>Ccrown</t>
+  </si>
+  <si>
+    <t>cc</t>
+  </si>
+  <si>
+    <t>ZR95_L</t>
+  </si>
+  <si>
+    <t>Kbot</t>
+  </si>
+  <si>
+    <t>f_O_in</t>
+  </si>
+  <si>
+    <t>soil_temp</t>
+  </si>
+  <si>
+    <t>PFT_type</t>
+  </si>
+  <si>
+    <t>stature_type</t>
+  </si>
+  <si>
+    <t>Urbana (US)</t>
+  </si>
+  <si>
+    <t>Kantola</t>
+  </si>
+  <si>
+    <t>MOD_PARAM_Kantola_Maize_Soy</t>
+  </si>
+  <si>
+    <t>2016-2020</t>
+  </si>
+  <si>
+    <t>[0 10 50 100 150 200 300 400 600 800 1000 1250 1500 1750 2000 2500 3000 3500 4000 4500 5000]</t>
+  </si>
+  <si>
+    <t>[0 0]</t>
+  </si>
+  <si>
+    <t>2009-2016</t>
+  </si>
+  <si>
+    <t>ExperimentalDescription</t>
+  </si>
+  <si>
+    <t>opt_TC_biochem</t>
+  </si>
+  <si>
+    <t>opt_crop</t>
+  </si>
+  <si>
+    <t>fX_conc_convention</t>
+  </si>
+  <si>
+    <t>keyword_add</t>
+  </si>
+  <si>
+    <t>rock_dist_data</t>
+  </si>
+  <si>
+    <t>rock_filepath</t>
+  </si>
+  <si>
+    <t>rock_type</t>
+  </si>
+  <si>
+    <t>soil</t>
+  </si>
+  <si>
+    <t>CEC_tot_in</t>
+  </si>
+  <si>
+    <t>MgCO3_in</t>
+  </si>
+  <si>
+    <t>CaCO3_in</t>
+  </si>
+  <si>
+    <t>Mg_in</t>
+  </si>
+  <si>
+    <t>Ca_in</t>
+  </si>
+  <si>
+    <t>K_in</t>
+  </si>
+  <si>
+    <t>Na_in</t>
+  </si>
+  <si>
+    <t>Si_in</t>
+  </si>
+  <si>
+    <t>Al_w_in</t>
+  </si>
+  <si>
+    <t>f_CEC_in</t>
+  </si>
   <si>
     <t>M_rock_in</t>
   </si>
   <si>
+    <t>mineral</t>
+  </si>
+  <si>
+    <t>rock_f_in</t>
+  </si>
+  <si>
     <t>rho_rock</t>
   </si>
   <si>
+    <t>d_in</t>
+  </si>
+  <si>
+    <t>psd_in</t>
+  </si>
+  <si>
+    <t>SSA_in</t>
+  </si>
+  <si>
+    <t>diss_f_original</t>
+  </si>
+  <si>
     <t>diss_f</t>
   </si>
   <si>
     <t>Alk_rain</t>
   </si>
   <si>
-    <t>Number</t>
-  </si>
-  <si>
-    <t>Location</t>
-  </si>
-  <si>
-    <t>Lat</t>
-  </si>
-  <si>
-    <t>Lon</t>
-  </si>
-  <si>
-    <t>Ccrown</t>
-  </si>
-  <si>
-    <t>Year</t>
-  </si>
-  <si>
-    <t>PH</t>
-  </si>
-  <si>
-    <t>rsd</t>
-  </si>
-  <si>
-    <t>keyword_add</t>
-  </si>
-  <si>
-    <t>soil</t>
-  </si>
-  <si>
-    <t>mineral</t>
-  </si>
-  <si>
-    <t>Cbare</t>
-  </si>
-  <si>
-    <t>Pcla</t>
-  </si>
-  <si>
-    <t>Psan</t>
-  </si>
-  <si>
-    <t>Porg</t>
-  </si>
-  <si>
-    <t>Zs</t>
-  </si>
-  <si>
-    <t>Zbio</t>
-  </si>
-  <si>
-    <t>MgCO3_in</t>
-  </si>
-  <si>
-    <t>SSA_in</t>
-  </si>
-  <si>
-    <t>rock_f_in</t>
-  </si>
-  <si>
-    <t>d_in</t>
-  </si>
-  <si>
-    <t>psd_in</t>
-  </si>
-  <si>
-    <t>ZR95_L</t>
-  </si>
-  <si>
-    <t>opt_TC_biochem</t>
-  </si>
-  <si>
-    <t>opt_crop</t>
-  </si>
-  <si>
-    <t>Mg_in</t>
-  </si>
-  <si>
-    <t>Si_in</t>
-  </si>
-  <si>
-    <t>rock_type</t>
-  </si>
-  <si>
-    <t>fX_conc_convention</t>
-  </si>
-  <si>
-    <t>Ca_in</t>
-  </si>
-  <si>
-    <t>K_in</t>
-  </si>
-  <si>
-    <t>Na_in</t>
-  </si>
-  <si>
-    <t>Al_w_in</t>
-  </si>
-  <si>
-    <t>rock_dist_data</t>
-  </si>
-  <si>
-    <t>rock_filepath</t>
-  </si>
-  <si>
-    <t>f_CEC_in</t>
-  </si>
-  <si>
-    <t>Kbot</t>
-  </si>
-  <si>
-    <t>f_O_in</t>
-  </si>
-  <si>
-    <t>soil_temp</t>
-  </si>
-  <si>
-    <t>diss_f_original</t>
-  </si>
-  <si>
-    <t>CaCO3_in</t>
-  </si>
-  <si>
-    <t>Urbana (US)</t>
-  </si>
-  <si>
-    <t>Kantola</t>
-  </si>
-  <si>
-    <t>2016-2020</t>
+    <t>pH_DilutionFactor</t>
+  </si>
+  <si>
+    <t>crop_Beerling</t>
+  </si>
+  <si>
+    <t>blueridge_CDF_data.json</t>
+  </si>
+  <si>
+    <t>Blueridge</t>
   </si>
   <si>
     <t>silty loam</t>
   </si>
   <si>
-    <t>blueridge_CDF_data.json</t>
-  </si>
-  <si>
-    <t>cc</t>
-  </si>
-  <si>
-    <t>[0 10 50 100 150 200 300 400 600 800 1000 1250 1500 1750 2000 2500 3000 3500 4000 4500 5000]</t>
-  </si>
-  <si>
-    <t>MOD_PARAM</t>
-  </si>
-  <si>
-    <t>MOD_PARAM_Kantola_Maize_Soy</t>
-  </si>
-  <si>
-    <t>Blueridge</t>
+    <t>["albite", "ferroactinolite", "epidote", "chlorite","quartz","calcite"]</t>
+  </si>
+  <si>
+    <t>[0.233,0.119,0.178,0.34,0.09,0.026]</t>
+  </si>
+  <si>
+    <t>crop_Lewis</t>
+  </si>
+  <si>
+    <t>["albite", "ferroactinolite", "epidote", "chlorite","quartz"]</t>
+  </si>
+  <si>
+    <t>[0.196,0.116,0.256,0.363,0.052]</t>
   </si>
   <si>
     <t>crop_control</t>
   </si>
   <si>
-    <t>t_res</t>
-  </si>
-  <si>
-    <t>ExperimentFullName</t>
-  </si>
-  <si>
-    <t>ExperimentalDescription</t>
-  </si>
-  <si>
-    <t>NumberOfDays</t>
-  </si>
-  <si>
-    <t>PFT_type</t>
-  </si>
-  <si>
-    <t>stature_type</t>
+    <t>pretreatment</t>
+  </si>
+  <si>
+    <t>crop_calcite</t>
+  </si>
+  <si>
+    <t>["calcite"]</t>
   </si>
   <si>
     <t>[1]</t>
-  </si>
-  <si>
-    <t>[0 0]</t>
-  </si>
-  <si>
-    <t>CEC_tot_in</t>
-  </si>
-  <si>
-    <t>pretreatment</t>
-  </si>
-  <si>
-    <t>2009-2016</t>
-  </si>
-  <si>
-    <t>["albite", "ferroactinolite", "epidote", "chlorite","quartz"]</t>
-  </si>
-  <si>
-    <t>[0.196,0.116,0.256,0.363,0.052]</t>
-  </si>
-  <si>
-    <t>[0.233,0.119,0.178,0.34,0.09,0.026]</t>
-  </si>
-  <si>
-    <t>["albite", "ferroactinolite", "epidote", "chlorite","quartz","calcite"]</t>
-  </si>
-  <si>
-    <t>crop_Beerling</t>
-  </si>
-  <si>
-    <t>crop_Lewis</t>
-  </si>
-  <si>
-    <t>crop_calcite</t>
-  </si>
-  <si>
-    <t>["calcite"]</t>
-  </si>
-  <si>
-    <t>pH_DilutionFactor</t>
   </si>
 </sst>
 </file>
@@ -711,7 +708,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7CD89003-D51E-46FB-A15B-91DFDAA3BEF6}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Y12"/>
   <sheetFormatPr defaultColWidth="8.68359375" defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
@@ -725,97 +722,98 @@
     <col min="8" max="8" width="15" style="2" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="12.41796875" style="2" customWidth="1"/>
     <col min="10" max="10" width="9.1015625" style="2" customWidth="1"/>
-    <col min="11" max="11" width="8.68359375" style="2"/>
+    <col min="11" max="11" width="8.68359375" style="2" customWidth="1"/>
     <col min="12" max="12" width="10" style="2" customWidth="1"/>
-    <col min="13" max="14" width="8.68359375" style="2"/>
+    <col min="13" max="14" width="8.68359375" style="2" customWidth="1"/>
     <col min="15" max="15" width="112.41796875" style="2" customWidth="1"/>
     <col min="16" max="16" width="9.89453125" style="2" customWidth="1"/>
     <col min="17" max="17" width="8.5234375" style="2" customWidth="1"/>
     <col min="18" max="18" width="9.5234375" style="2" customWidth="1"/>
     <col min="19" max="19" width="8.5234375" style="2" customWidth="1"/>
     <col min="20" max="20" width="12.5234375" style="2" customWidth="1"/>
-    <col min="21" max="22" width="8.68359375" style="2"/>
+    <col min="21" max="22" width="8.68359375" style="2" customWidth="1"/>
     <col min="23" max="23" width="10.3125" style="2" customWidth="1"/>
-    <col min="24" max="24" width="8.68359375" style="2"/>
+    <col min="24" max="24" width="8.68359375" style="2" customWidth="1"/>
     <col min="25" max="25" width="11.68359375" style="2" customWidth="1"/>
-    <col min="26" max="16384" width="8.68359375" style="2"/>
+    <col min="26" max="26" width="8.68359375" style="2" customWidth="1"/>
+    <col min="27" max="16384" width="8.68359375" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:25" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="15" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="16" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="17" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="15" t="s">
-        <v>57</v>
-      </c>
-      <c r="C1" s="16" t="s">
+      <c r="F1" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="D1" s="17" t="s">
+      <c r="G1" s="16" t="s">
         <v>6</v>
       </c>
-      <c r="E1" s="17" t="s">
+      <c r="H1" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="F1" s="13" t="s">
-        <v>52</v>
-      </c>
-      <c r="G1" s="16" t="s">
-        <v>56</v>
-      </c>
-      <c r="H1" s="17" t="s">
-        <v>59</v>
-      </c>
       <c r="I1" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="J1" s="18" t="s">
+      <c r="K1" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="K1" s="6" t="s">
+      <c r="L1" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="L1" s="6" t="s">
+      <c r="M1" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="M1" s="6" t="s">
+      <c r="R1" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="N1" s="6" t="s">
+      <c r="S1" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="O1" s="6" t="s">
+      <c r="T1" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="P1" s="6" t="s">
+      <c r="U1" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="Q1" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="R1" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="S1" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="T1" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="U1" s="6" t="s">
-        <v>40</v>
-      </c>
       <c r="V1" s="6" t="s">
-        <v>41</v>
+        <v>21</v>
       </c>
       <c r="W1" s="6" t="s">
-        <v>42</v>
+        <v>22</v>
       </c>
       <c r="X1" s="6" t="s">
-        <v>60</v>
+        <v>23</v>
       </c>
       <c r="Y1" s="6" t="s">
-        <v>61</v>
+        <v>24</v>
       </c>
     </row>
     <row r="2" spans="1:25" x14ac:dyDescent="0.55000000000000004">
@@ -823,10 +821,10 @@
         <v>3</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>45</v>
+        <v>25</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>46</v>
+        <v>26</v>
       </c>
       <c r="D2" s="9">
         <v>40.062778000000002</v>
@@ -835,7 +833,7 @@
         <v>-88.196111000000002</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>53</v>
+        <v>27</v>
       </c>
       <c r="G2" s="2">
         <v>6</v>
@@ -844,7 +842,7 @@
         <v>1825</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>47</v>
+        <v>28</v>
       </c>
       <c r="J2" s="19">
         <v>6.1</v>
@@ -862,7 +860,7 @@
         <v>2.5000000000000001E-2</v>
       </c>
       <c r="O2" s="14" t="s">
-        <v>51</v>
+        <v>29</v>
       </c>
       <c r="P2" s="2">
         <v>300</v>
@@ -871,25 +869,21 @@
         <v>1</v>
       </c>
       <c r="R2" s="2" t="s">
-        <v>63</v>
+        <v>30</v>
       </c>
       <c r="S2" s="2">
         <v>2</v>
       </c>
-      <c r="T2"/>
-      <c r="U2"/>
-      <c r="V2"/>
-      <c r="W2"/>
     </row>
     <row r="3" spans="1:25" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" s="2">
         <v>4</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>45</v>
+        <v>25</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>46</v>
+        <v>26</v>
       </c>
       <c r="D3" s="9">
         <v>40.062778000000002</v>
@@ -898,7 +892,7 @@
         <v>-88.196111000000002</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>53</v>
+        <v>27</v>
       </c>
       <c r="G3" s="2">
         <v>6</v>
@@ -907,7 +901,7 @@
         <v>1825</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>47</v>
+        <v>28</v>
       </c>
       <c r="J3" s="19">
         <v>6.1</v>
@@ -925,7 +919,7 @@
         <v>2.5000000000000001E-2</v>
       </c>
       <c r="O3" s="14" t="s">
-        <v>51</v>
+        <v>29</v>
       </c>
       <c r="P3" s="2">
         <v>300</v>
@@ -934,25 +928,21 @@
         <v>1</v>
       </c>
       <c r="R3" s="2" t="s">
-        <v>63</v>
+        <v>30</v>
       </c>
       <c r="S3" s="2">
         <v>2</v>
       </c>
-      <c r="T3"/>
-      <c r="U3"/>
-      <c r="V3"/>
-      <c r="W3"/>
     </row>
     <row r="4" spans="1:25" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="2">
         <v>5</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>45</v>
+        <v>25</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>46</v>
+        <v>26</v>
       </c>
       <c r="D4" s="9">
         <v>40.062778000000002</v>
@@ -961,7 +951,7 @@
         <v>-88.196111000000002</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>53</v>
+        <v>27</v>
       </c>
       <c r="G4" s="2">
         <v>6</v>
@@ -970,7 +960,7 @@
         <v>1825</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>66</v>
+        <v>31</v>
       </c>
       <c r="J4" s="19">
         <v>6.1</v>
@@ -988,7 +978,7 @@
         <v>2.5000000000000001E-2</v>
       </c>
       <c r="O4" s="14" t="s">
-        <v>51</v>
+        <v>29</v>
       </c>
       <c r="P4" s="2">
         <v>300</v>
@@ -997,25 +987,21 @@
         <v>1</v>
       </c>
       <c r="R4" s="2" t="s">
-        <v>63</v>
+        <v>30</v>
       </c>
       <c r="S4" s="2">
         <v>2</v>
       </c>
-      <c r="T4"/>
-      <c r="U4"/>
-      <c r="V4"/>
-      <c r="W4"/>
     </row>
     <row r="5" spans="1:25" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="2">
         <v>6</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>45</v>
+        <v>25</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>46</v>
+        <v>26</v>
       </c>
       <c r="D5" s="9">
         <v>40.062778000000002</v>
@@ -1024,7 +1010,7 @@
         <v>-88.196111000000002</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>53</v>
+        <v>27</v>
       </c>
       <c r="G5" s="2">
         <v>6</v>
@@ -1033,7 +1019,7 @@
         <v>1825</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>66</v>
+        <v>31</v>
       </c>
       <c r="J5" s="19">
         <v>6.1</v>
@@ -1051,7 +1037,7 @@
         <v>2.5000000000000001E-2</v>
       </c>
       <c r="O5" s="14" t="s">
-        <v>51</v>
+        <v>29</v>
       </c>
       <c r="P5" s="2">
         <v>300</v>
@@ -1060,25 +1046,21 @@
         <v>1</v>
       </c>
       <c r="R5" s="2" t="s">
-        <v>63</v>
+        <v>30</v>
       </c>
       <c r="S5" s="2">
         <v>2</v>
       </c>
-      <c r="T5"/>
-      <c r="U5"/>
-      <c r="V5"/>
-      <c r="W5"/>
     </row>
     <row r="6" spans="1:25" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" s="2">
         <v>7</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>45</v>
+        <v>25</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>46</v>
+        <v>26</v>
       </c>
       <c r="D6" s="9">
         <v>40.062778000000002</v>
@@ -1087,7 +1069,7 @@
         <v>-88.196111000000002</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>53</v>
+        <v>27</v>
       </c>
       <c r="G6" s="2">
         <v>6</v>
@@ -1096,7 +1078,7 @@
         <v>1825</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>47</v>
+        <v>28</v>
       </c>
       <c r="J6" s="19">
         <v>6.1</v>
@@ -1114,7 +1096,7 @@
         <v>2.5000000000000001E-2</v>
       </c>
       <c r="O6" s="14" t="s">
-        <v>51</v>
+        <v>29</v>
       </c>
       <c r="P6" s="2">
         <v>300</v>
@@ -1123,21 +1105,11 @@
         <v>1</v>
       </c>
       <c r="R6" s="2" t="s">
-        <v>63</v>
+        <v>30</v>
       </c>
       <c r="S6" s="2">
         <v>2</v>
       </c>
-      <c r="T6"/>
-      <c r="U6"/>
-      <c r="V6"/>
-      <c r="W6"/>
-    </row>
-    <row r="7" spans="1:25" x14ac:dyDescent="0.55000000000000004">
-      <c r="J7"/>
-    </row>
-    <row r="8" spans="1:25" x14ac:dyDescent="0.55000000000000004">
-      <c r="J8"/>
     </row>
     <row r="9" spans="1:25" x14ac:dyDescent="0.55000000000000004">
       <c r="S9" s="9"/>
@@ -1150,13 +1122,13 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
+  <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D139F640-0076-4304-86A9-B1EEDC96C211}">
-  <dimension ref="A1:AH6"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:AI6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="10.1015625" customWidth="1"/>
@@ -1185,36 +1157,36 @@
     <col min="36" max="36" width="11.3125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:34" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:35" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="10" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="11" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="12" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="10" t="s">
-        <v>57</v>
-      </c>
-      <c r="C1" s="11" t="s">
-        <v>5</v>
-      </c>
-      <c r="D1" s="12" t="s">
-        <v>6</v>
-      </c>
-      <c r="E1" s="12" t="s">
-        <v>7</v>
-      </c>
       <c r="F1" s="13" t="s">
-        <v>58</v>
+        <v>32</v>
       </c>
       <c r="G1" s="6" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="H1" s="6" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="I1" s="6" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="J1" s="5" t="s">
-        <v>12</v>
+        <v>36</v>
       </c>
       <c r="K1" s="5" t="s">
         <v>37</v>
@@ -1223,84 +1195,84 @@
         <v>38</v>
       </c>
       <c r="M1" s="5" t="s">
-        <v>31</v>
+        <v>39</v>
       </c>
       <c r="N1" s="5" t="s">
-        <v>13</v>
+        <v>40</v>
       </c>
       <c r="O1" s="5" t="s">
-        <v>64</v>
+        <v>41</v>
       </c>
       <c r="P1" s="5" t="s">
-        <v>21</v>
+        <v>42</v>
       </c>
       <c r="Q1" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="R1" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="R1" s="5" t="s">
-        <v>29</v>
-      </c>
       <c r="S1" s="5" t="s">
-        <v>33</v>
+        <v>45</v>
       </c>
       <c r="T1" s="5" t="s">
-        <v>34</v>
+        <v>46</v>
       </c>
       <c r="U1" s="5" t="s">
-        <v>35</v>
+        <v>47</v>
       </c>
       <c r="V1" s="5" t="s">
-        <v>30</v>
+        <v>48</v>
       </c>
       <c r="W1" s="5" t="s">
-        <v>36</v>
+        <v>49</v>
       </c>
       <c r="X1" s="5" t="s">
-        <v>39</v>
+        <v>50</v>
       </c>
       <c r="Y1" s="5" t="s">
-        <v>0</v>
+        <v>51</v>
       </c>
       <c r="Z1" s="5" t="s">
-        <v>14</v>
+        <v>52</v>
       </c>
       <c r="AA1" s="5" t="s">
-        <v>23</v>
+        <v>53</v>
       </c>
       <c r="AB1" s="5" t="s">
-        <v>1</v>
+        <v>54</v>
       </c>
       <c r="AC1" s="5" t="s">
-        <v>24</v>
+        <v>55</v>
       </c>
       <c r="AD1" s="5" t="s">
-        <v>25</v>
+        <v>56</v>
       </c>
       <c r="AE1" s="5" t="s">
-        <v>22</v>
+        <v>57</v>
       </c>
       <c r="AF1" s="5" t="s">
-        <v>43</v>
+        <v>58</v>
       </c>
       <c r="AG1" s="5" t="s">
-        <v>2</v>
+        <v>59</v>
       </c>
       <c r="AH1" s="5" t="s">
-        <v>3</v>
+        <v>60</v>
       </c>
       <c r="AI1" s="5" t="s">
-        <v>75</v>
+        <v>61</v>
       </c>
     </row>
-    <row r="2" spans="1:34" x14ac:dyDescent="0.55000000000000004">
+    <row r="2" spans="1:35" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" s="4">
         <v>3</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>45</v>
+        <v>25</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>46</v>
+        <v>26</v>
       </c>
       <c r="D2" s="9">
         <v>40.062778000000002</v>
@@ -1309,7 +1281,7 @@
         <v>-88.196111000000002</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>71</v>
+        <v>62</v>
       </c>
       <c r="G2" s="2">
         <v>1</v>
@@ -1318,25 +1290,25 @@
         <v>1</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>46</v>
+        <v>26</v>
       </c>
       <c r="J2" s="4">
         <v>1</v>
       </c>
       <c r="K2" t="s">
-        <v>46</v>
+        <v>26</v>
       </c>
       <c r="L2" t="s">
-        <v>49</v>
+        <v>63</v>
       </c>
       <c r="M2" t="s">
-        <v>54</v>
+        <v>64</v>
       </c>
       <c r="N2" t="s">
-        <v>48</v>
+        <v>65</v>
       </c>
       <c r="O2" s="7">
-        <v>8.6</v>
+        <v>13</v>
       </c>
       <c r="P2" s="7">
         <v>0</v>
@@ -1354,13 +1326,12 @@
         <v>0</v>
       </c>
       <c r="Z2" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="AA2" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="AB2">
-        <f t="shared" ref="AB2:AB3" si="0">3*1000000</f>
         <v>3000000</v>
       </c>
       <c r="AE2">
@@ -1373,18 +1344,18 @@
         <v>0</v>
       </c>
       <c r="AI2">
-        <v>2.5</v>
+        <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:34" x14ac:dyDescent="0.55000000000000004">
+    <row r="3" spans="1:35" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" s="4">
         <v>4</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>45</v>
+        <v>25</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>46</v>
+        <v>26</v>
       </c>
       <c r="D3" s="9">
         <v>40.062778000000002</v>
@@ -1393,7 +1364,7 @@
         <v>-88.196111000000002</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="G3" s="2">
         <v>1</v>
@@ -1402,25 +1373,25 @@
         <v>1</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>46</v>
+        <v>26</v>
       </c>
       <c r="J3" s="4">
         <v>1</v>
       </c>
       <c r="K3" t="s">
-        <v>46</v>
+        <v>26</v>
       </c>
       <c r="L3" t="s">
-        <v>49</v>
+        <v>63</v>
       </c>
       <c r="M3" t="s">
-        <v>54</v>
+        <v>64</v>
       </c>
       <c r="N3" t="s">
-        <v>48</v>
+        <v>65</v>
       </c>
       <c r="O3" s="7">
-        <v>8.6</v>
+        <v>13</v>
       </c>
       <c r="P3" s="7">
         <v>0</v>
@@ -1438,13 +1409,13 @@
         <v>0</v>
       </c>
       <c r="Z3" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="AA3" s="1" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="AB3">
-        <f t="shared" si="0"/>
+        <f>3*1000000</f>
         <v>3000000</v>
       </c>
       <c r="AE3">
@@ -1457,18 +1428,18 @@
         <v>0</v>
       </c>
       <c r="AI3">
-        <v>2.5</v>
+        <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:34" x14ac:dyDescent="0.55000000000000004">
+    <row r="4" spans="1:35" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="4">
         <v>5</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>45</v>
+        <v>25</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>46</v>
+        <v>26</v>
       </c>
       <c r="D4" s="9">
         <v>40.062778000000002</v>
@@ -1477,7 +1448,7 @@
         <v>-88.196111000000002</v>
       </c>
       <c r="F4" t="s">
-        <v>55</v>
+        <v>71</v>
       </c>
       <c r="G4" s="2">
         <v>1</v>
@@ -1486,19 +1457,19 @@
         <v>1</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>46</v>
+        <v>26</v>
       </c>
       <c r="J4" s="4">
         <v>1</v>
       </c>
       <c r="K4" t="s">
-        <v>46</v>
+        <v>26</v>
       </c>
       <c r="N4" t="s">
-        <v>48</v>
+        <v>65</v>
       </c>
       <c r="O4" s="7">
-        <v>8.6</v>
+        <v>13</v>
       </c>
       <c r="P4" s="7">
         <v>0</v>
@@ -1520,18 +1491,18 @@
         <v>0</v>
       </c>
       <c r="AI4">
-        <v>2.5</v>
+        <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:34" x14ac:dyDescent="0.55000000000000004">
+    <row r="5" spans="1:35" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="4">
         <v>6</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>45</v>
+        <v>25</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>46</v>
+        <v>26</v>
       </c>
       <c r="D5" s="9">
         <v>40.062778000000002</v>
@@ -1540,28 +1511,28 @@
         <v>-88.196111000000002</v>
       </c>
       <c r="F5" t="s">
+        <v>72</v>
+      </c>
+      <c r="G5" s="2">
+        <v>1</v>
+      </c>
+      <c r="H5" s="2">
+        <v>1</v>
+      </c>
+      <c r="I5" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="J5" s="4">
+        <v>1</v>
+      </c>
+      <c r="K5" t="s">
+        <v>26</v>
+      </c>
+      <c r="N5" t="s">
         <v>65</v>
       </c>
-      <c r="G5" s="2">
-        <v>1</v>
-      </c>
-      <c r="H5" s="2">
-        <v>1</v>
-      </c>
-      <c r="I5" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="J5" s="4">
-        <v>1</v>
-      </c>
-      <c r="K5" t="s">
-        <v>46</v>
-      </c>
-      <c r="N5" t="s">
-        <v>48</v>
-      </c>
       <c r="O5" s="7">
-        <v>8.6</v>
+        <v>13</v>
       </c>
       <c r="P5" s="7">
         <v>0</v>
@@ -1583,18 +1554,18 @@
         <v>0</v>
       </c>
       <c r="AI5">
-        <v>2.5</v>
+        <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:34" x14ac:dyDescent="0.55000000000000004">
+    <row r="6" spans="1:35" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" s="4">
         <v>7</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>45</v>
+        <v>25</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>46</v>
+        <v>26</v>
       </c>
       <c r="D6" s="9">
         <v>40.062778000000002</v>
@@ -1612,25 +1583,25 @@
         <v>1</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>46</v>
+        <v>26</v>
       </c>
       <c r="J6" s="4">
         <v>1</v>
       </c>
       <c r="K6" t="s">
-        <v>46</v>
+        <v>26</v>
       </c>
       <c r="L6" t="s">
-        <v>49</v>
+        <v>63</v>
       </c>
       <c r="M6" t="s">
-        <v>54</v>
+        <v>64</v>
       </c>
       <c r="N6" t="s">
-        <v>48</v>
+        <v>65</v>
       </c>
       <c r="O6" s="7">
-        <v>8.6</v>
+        <v>13</v>
       </c>
       <c r="P6" s="7">
         <v>0</v>
@@ -1651,11 +1622,10 @@
         <v>74</v>
       </c>
       <c r="AA6" s="1" t="s">
-        <v>62</v>
+        <v>75</v>
       </c>
       <c r="AB6">
-        <f t="shared" ref="AB6" si="1">3*1000000</f>
-        <v>3000000</v>
+        <v>2710000</v>
       </c>
       <c r="AE6">
         <v>1.02</v>
@@ -1667,311 +1637,11 @@
         <v>0</v>
       </c>
       <c r="AI6">
-        <v>2.5</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
+  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
-</file>
-
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <SharedWithUsers xmlns="155627c1-0cf9-4357-bbd5-48008c93d75a">
-      <UserInfo>
-        <DisplayName>Jones, Gregory</DisplayName>
-        <AccountId>12</AccountId>
-        <AccountType/>
-      </UserInfo>
-    </SharedWithUsers>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="65a37cd7-3d23-4aec-ad96-417b75cab311">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="155627c1-0cf9-4357-bbd5-48008c93d75a" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100BA25395398D53143824DAEC78DD9561A" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="20ccdcc7d59f2619f731219bc917c622">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="65a37cd7-3d23-4aec-ad96-417b75cab311" xmlns:ns3="155627c1-0cf9-4357-bbd5-48008c93d75a" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="e26a2ebc3a37e9b8f4c1fbd5093d1833" ns2:_="" ns3:_="">
-    <xsd:import namespace="65a37cd7-3d23-4aec-ad96-417b75cab311"/>
-    <xsd:import namespace="155627c1-0cf9-4357-bbd5-48008c93d75a"/>
-    <xsd:element name="properties">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element name="documentManagement">
-            <xsd:complexType>
-              <xsd:all>
-                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
-                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
-                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
-              </xsd:all>
-            </xsd:complexType>
-          </xsd:element>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="65a37cd7-3d23-4aec-ad96-417b75cab311" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="10" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="11" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="15" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="74661dae-d6df-48fc-a54e-a577d2899e9c" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="17" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="18" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="19" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="20" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaLengthInSeconds" ma:index="21" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Unknown"/>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="155627c1-0cf9-4357-bbd5-48008c93d75a" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="SharedWithUsers" ma:index="12" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:UserMulti">
-            <xsd:sequence>
-              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
-                <xsd:complexType>
-                  <xsd:sequence>
-                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
-                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
-                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
-                  </xsd:sequence>
-                </xsd:complexType>
-              </xsd:element>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="SharedWithDetails" ma:index="13" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="TaxCatchAll" ma:index="16" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{7e2022d3-544c-4e93-95c6-8b7474f5c6b3}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="155627c1-0cf9-4357-bbd5-48008c93d75a">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:MultiChoiceLookup">
-            <xsd:sequence>
-              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
-    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
-    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
-    <xsd:element name="coreProperties" type="CT_coreProperties"/>
-    <xsd:complexType name="CT_coreProperties">
-      <xsd:all>
-        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
-        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
-          <xsd:annotation>
-            <xsd:documentation>
-                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
-                    </xsd:documentation>
-          </xsd:annotation>
-        </xsd:element>
-        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-      </xsd:all>
-    </xsd:complexType>
-  </xsd:schema>
-  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
-    <xs:element name="Person">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:DisplayName" minOccurs="0"/>
-          <xs:element ref="pc:AccountId" minOccurs="0"/>
-          <xs:element ref="pc:AccountType" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="DisplayName" type="xs:string"/>
-    <xs:element name="AccountId" type="xs:string"/>
-    <xs:element name="AccountType" type="xs:string"/>
-    <xs:element name="BDCAssociatedEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-        <xs:attribute ref="pc:EntityNamespace"/>
-        <xs:attribute ref="pc:EntityName"/>
-        <xs:attribute ref="pc:SystemInstanceName"/>
-        <xs:attribute ref="pc:AssociationName"/>
-      </xs:complexType>
-    </xs:element>
-    <xs:attribute name="EntityNamespace" type="xs:string"/>
-    <xs:attribute name="EntityName" type="xs:string"/>
-    <xs:attribute name="SystemInstanceName" type="xs:string"/>
-    <xs:attribute name="AssociationName" type="xs:string"/>
-    <xs:element name="BDCEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
-          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
-          <xs:element ref="pc:EntityId1" minOccurs="0"/>
-          <xs:element ref="pc:EntityId2" minOccurs="0"/>
-          <xs:element ref="pc:EntityId3" minOccurs="0"/>
-          <xs:element ref="pc:EntityId4" minOccurs="0"/>
-          <xs:element ref="pc:EntityId5" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="EntityDisplayName" type="xs:string"/>
-    <xs:element name="EntityInstanceReference" type="xs:string"/>
-    <xs:element name="EntityId1" type="xs:string"/>
-    <xs:element name="EntityId2" type="xs:string"/>
-    <xs:element name="EntityId3" type="xs:string"/>
-    <xs:element name="EntityId4" type="xs:string"/>
-    <xs:element name="EntityId5" type="xs:string"/>
-    <xs:element name="Terms">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermInfo">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermName" minOccurs="0"/>
-          <xs:element ref="pc:TermId" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermName" type="xs:string"/>
-    <xs:element name="TermId" type="xs:string"/>
-  </xs:schema>
-</ct:contentTypeSchema>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CA802978-8DC2-44C2-8CFD-840D40C88D7C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="155627c1-0cf9-4357-bbd5-48008c93d75a"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="65a37cd7-3d23-4aec-ad96-417b75cab311"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AAA6EAB6-7EA4-41C9-A63C-13457F927A01}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="65a37cd7-3d23-4aec-ad96-417b75cab311"/>
-    <ds:schemaRef ds:uri="155627c1-0cf9-4357-bbd5-48008c93d75a"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C4807397-6038-423A-9DD2-E48912B9B2FD}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>